<commit_message>
Improved code and updated files after first revision
</commit_message>
<xml_diff>
--- a/outputFiles/trialValidity.xlsx
+++ b/outputFiles/trialValidity.xlsx
@@ -562,30 +562,30 @@
   <dimension ref="A1:X104"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="17.8046875" customWidth="true"/>
-    <col min="2" max="2" width="6.07421875" customWidth="true"/>
-    <col min="3" max="3" width="14.2578125" customWidth="true"/>
-    <col min="4" max="4" width="5.16796875" customWidth="true"/>
-    <col min="5" max="5" width="9.89453125" customWidth="true"/>
-    <col min="6" max="6" width="11.2578125" customWidth="true"/>
-    <col min="7" max="7" width="6.984375" customWidth="true"/>
-    <col min="8" max="8" width="6.53125" customWidth="true"/>
-    <col min="9" max="9" width="14.89453125" customWidth="true"/>
-    <col min="10" max="10" width="15.7109375" customWidth="true"/>
-    <col min="11" max="11" width="10.53125" customWidth="true"/>
-    <col min="12" max="12" width="9.2578125" customWidth="true"/>
-    <col min="13" max="13" width="12.07421875" customWidth="true"/>
-    <col min="14" max="14" width="11.984375" customWidth="true"/>
-    <col min="15" max="15" width="12.2578125" customWidth="true"/>
-    <col min="16" max="16" width="10.7109375" customWidth="true"/>
-    <col min="17" max="17" width="10.984375" customWidth="true"/>
-    <col min="18" max="18" width="18.44140625" customWidth="true"/>
-    <col min="19" max="19" width="17.16796875" customWidth="true"/>
-    <col min="20" max="20" width="19.984375" customWidth="true"/>
-    <col min="21" max="21" width="19.89453125" customWidth="true"/>
-    <col min="22" max="22" width="20.16796875" customWidth="true"/>
-    <col min="23" max="23" width="18.62109375" customWidth="true"/>
-    <col min="24" max="24" width="18.89453125" customWidth="true"/>
+    <col min="1" max="1" width="17.37890625" customWidth="true"/>
+    <col min="2" max="2" width="5.82421875" customWidth="true"/>
+    <col min="3" max="3" width="14.15625" customWidth="true"/>
+    <col min="4" max="4" width="5.15625" customWidth="true"/>
+    <col min="5" max="5" width="9.6015625" customWidth="true"/>
+    <col min="6" max="6" width="10.93359375" customWidth="true"/>
+    <col min="7" max="7" width="6.7109375" customWidth="true"/>
+    <col min="8" max="8" width="6.48828125" customWidth="true"/>
+    <col min="9" max="9" width="14.7109375" customWidth="true"/>
+    <col min="10" max="10" width="15.48828125" customWidth="true"/>
+    <col min="11" max="11" width="10.37890625" customWidth="true"/>
+    <col min="12" max="12" width="9.15625" customWidth="true"/>
+    <col min="13" max="13" width="11.93359375" customWidth="true"/>
+    <col min="14" max="14" width="11.82421875" customWidth="true"/>
+    <col min="15" max="15" width="12.046875" customWidth="true"/>
+    <col min="16" max="16" width="10.6015625" customWidth="true"/>
+    <col min="17" max="17" width="10.82421875" customWidth="true"/>
+    <col min="18" max="18" width="18.26953125" customWidth="true"/>
+    <col min="19" max="19" width="17.046875" customWidth="true"/>
+    <col min="20" max="20" width="19.82421875" customWidth="true"/>
+    <col min="21" max="21" width="19.7109375" customWidth="true"/>
+    <col min="22" max="22" width="19.93359375" customWidth="true"/>
+    <col min="23" max="23" width="18.48828125" customWidth="true"/>
+    <col min="24" max="24" width="18.7109375" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1221,13 +1221,13 @@
         <v>0</v>
       </c>
       <c r="N9" s="0">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O9" s="0">
         <v>27</v>
       </c>
       <c r="P9" s="0">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Q9" s="0">
         <v>25</v>
@@ -1387,7 +1387,7 @@
         <v>32</v>
       </c>
       <c r="T11" s="0">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="U11" s="0">
         <v>15</v>
@@ -1618,7 +1618,7 @@
         <v>20</v>
       </c>
       <c r="W14" s="0">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="X14" s="0">
         <v>20</v>
@@ -1905,7 +1905,7 @@
         <v>43</v>
       </c>
       <c r="T18" s="0">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="U18" s="0">
         <v>8</v>
@@ -2201,7 +2201,7 @@
         <v>41</v>
       </c>
       <c r="T22" s="0">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="U22" s="0">
         <v>0</v>
@@ -2633,7 +2633,7 @@
         <v>11</v>
       </c>
       <c r="P28" s="0">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Q28" s="0">
         <v>12</v>
@@ -2775,7 +2775,7 @@
         <v>17</v>
       </c>
       <c r="N30" s="0">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O30" s="0">
         <v>0</v>
@@ -2846,7 +2846,7 @@
         <v>13</v>
       </c>
       <c r="M31" s="0">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="N31" s="0">
         <v>12</v>
@@ -2947,7 +2947,7 @@
         <v>0</v>
       </c>
       <c r="V32" s="0">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="W32" s="0">
         <v>28</v>
@@ -3299,7 +3299,7 @@
         <v>23</v>
       </c>
       <c r="P37" s="0">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Q37" s="0">
         <v>15</v>
@@ -3438,7 +3438,7 @@
         <v>38</v>
       </c>
       <c r="M39" s="0">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="N39" s="0">
         <v>8</v>
@@ -3589,7 +3589,7 @@
         <v>0</v>
       </c>
       <c r="N41" s="0">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O41" s="0">
         <v>21</v>
@@ -3808,7 +3808,7 @@
         <v>29</v>
       </c>
       <c r="M44" s="0">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="N44" s="0">
         <v>12</v>
@@ -4199,7 +4199,7 @@
         <v>36</v>
       </c>
       <c r="T49" s="0">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="U49" s="0">
         <v>0</v>
@@ -4208,7 +4208,7 @@
         <v>11</v>
       </c>
       <c r="W49" s="0">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="X49" s="0">
         <v>30</v>
@@ -4412,7 +4412,7 @@
         <v>23</v>
       </c>
       <c r="Q52" s="0">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="R52" s="0">
         <v>0</v>
@@ -4643,7 +4643,7 @@
         <v>34</v>
       </c>
       <c r="T55" s="0">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="U55" s="0">
         <v>12</v>
@@ -5013,13 +5013,13 @@
         <v>40</v>
       </c>
       <c r="T60" s="0">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="U60" s="0">
         <v>12</v>
       </c>
       <c r="V60" s="0">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="W60" s="0">
         <v>23</v>
@@ -5140,7 +5140,7 @@
         <v>18</v>
       </c>
       <c r="M62" s="0">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="N62" s="0">
         <v>10</v>
@@ -5205,7 +5205,7 @@
         <v>55</v>
       </c>
       <c r="J63" s="0">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="K63" s="0">
         <v>32</v>
@@ -5226,7 +5226,7 @@
         <v>25</v>
       </c>
       <c r="Q63" s="0">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="R63" s="0">
         <v>0</v>
@@ -5501,7 +5501,7 @@
         <v>60</v>
       </c>
       <c r="J67" s="0">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="K67" s="0">
         <v>0</v>
@@ -5723,7 +5723,7 @@
         <v>53</v>
       </c>
       <c r="J70" s="0">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="K70" s="0">
         <v>46</v>
@@ -5883,7 +5883,7 @@
         <v>13</v>
       </c>
       <c r="N72" s="0">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O72" s="0">
         <v>13</v>
@@ -6111,7 +6111,7 @@
         <v>14</v>
       </c>
       <c r="P75" s="0">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Q75" s="0">
         <v>10</v>
@@ -6407,7 +6407,7 @@
         <v>28</v>
       </c>
       <c r="P79" s="0">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Q79" s="0">
         <v>12</v>
@@ -6996,7 +6996,7 @@
         <v>21</v>
       </c>
       <c r="O87" s="0">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="P87" s="0">
         <v>9</v>
@@ -7215,13 +7215,13 @@
         <v>9</v>
       </c>
       <c r="N90" s="0">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O90" s="0">
         <v>15</v>
       </c>
       <c r="P90" s="0">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="Q90" s="0">
         <v>23</v>
@@ -7582,7 +7582,7 @@
         <v>35</v>
       </c>
       <c r="M95" s="0">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="N95" s="0">
         <v>16</v>
@@ -7865,7 +7865,7 @@
         <v>4855</v>
       </c>
       <c r="J99" s="0">
-        <v>366</v>
+        <v>348</v>
       </c>
       <c r="K99" s="0">
         <v>2186</v>
@@ -7874,19 +7874,19 @@
         <v>1449</v>
       </c>
       <c r="M99" s="0">
-        <v>730</v>
+        <v>700</v>
       </c>
       <c r="N99" s="0">
-        <v>643</v>
+        <v>613</v>
       </c>
       <c r="O99" s="0">
-        <v>686</v>
+        <v>680</v>
       </c>
       <c r="P99" s="0">
-        <v>596</v>
+        <v>560</v>
       </c>
       <c r="Q99" s="0">
-        <v>776</v>
+        <v>764</v>
       </c>
       <c r="R99" s="0">
         <v>795</v>
@@ -7895,16 +7895,16 @@
         <v>1090</v>
       </c>
       <c r="T99" s="0">
-        <v>209</v>
+        <v>173</v>
       </c>
       <c r="U99" s="0">
         <v>184</v>
       </c>
       <c r="V99" s="0">
-        <v>324</v>
+        <v>312</v>
       </c>
       <c r="W99" s="0">
-        <v>357</v>
+        <v>345</v>
       </c>
       <c r="X99" s="0">
         <v>712</v>
@@ -7935,7 +7935,7 @@
         <v>2459</v>
       </c>
       <c r="J100" s="0">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="K100" s="0">
         <v>1358</v>
@@ -7944,19 +7944,19 @@
         <v>953</v>
       </c>
       <c r="M100" s="0">
-        <v>394</v>
+        <v>370</v>
       </c>
       <c r="N100" s="0">
-        <v>394</v>
+        <v>376</v>
       </c>
       <c r="O100" s="0">
-        <v>477</v>
+        <v>471</v>
       </c>
       <c r="P100" s="0">
-        <v>389</v>
+        <v>359</v>
       </c>
       <c r="Q100" s="0">
-        <v>518</v>
+        <v>506</v>
       </c>
       <c r="R100" s="0">
         <v>140</v>
@@ -7965,13 +7965,13 @@
         <v>175</v>
       </c>
       <c r="T100" s="0">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="U100" s="0">
         <v>42</v>
       </c>
       <c r="V100" s="0">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="W100" s="0">
         <v>70</v>
@@ -8005,7 +8005,7 @@
         <v>2396</v>
       </c>
       <c r="J101" s="0">
-        <v>285</v>
+        <v>273</v>
       </c>
       <c r="K101" s="0">
         <v>828</v>
@@ -8014,16 +8014,16 @@
         <v>496</v>
       </c>
       <c r="M101" s="0">
-        <v>336</v>
+        <v>330</v>
       </c>
       <c r="N101" s="0">
-        <v>249</v>
+        <v>237</v>
       </c>
       <c r="O101" s="0">
         <v>209</v>
       </c>
       <c r="P101" s="0">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="Q101" s="0">
         <v>258</v>
@@ -8035,16 +8035,16 @@
         <v>915</v>
       </c>
       <c r="T101" s="0">
-        <v>169</v>
+        <v>139</v>
       </c>
       <c r="U101" s="0">
         <v>142</v>
       </c>
       <c r="V101" s="0">
-        <v>279</v>
+        <v>273</v>
       </c>
       <c r="W101" s="0">
-        <v>287</v>
+        <v>275</v>
       </c>
       <c r="X101" s="0">
         <v>607</v>
@@ -8077,7 +8077,7 @@
         <v>90</v>
       </c>
       <c r="J102" s="0">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="K102" s="0">
         <v>61</v>
@@ -8086,19 +8086,19 @@
         <v>61</v>
       </c>
       <c r="M102" s="0">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="N102" s="0">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="O102" s="0">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="P102" s="0">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="Q102" s="0">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="R102" s="0">
         <v>29</v>
@@ -8107,13 +8107,13 @@
         <v>30</v>
       </c>
       <c r="T102" s="0">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="U102" s="0">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="V102" s="0">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="W102" s="0">
         <v>21</v>
@@ -8158,19 +8158,19 @@
         <v>40</v>
       </c>
       <c r="M103" s="0">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="N103" s="0">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="O103" s="0">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="P103" s="0">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="Q103" s="0">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="R103" s="0">
         <v>5</v>
@@ -8185,7 +8185,7 @@
         <v>4</v>
       </c>
       <c r="V103" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="W103" s="0">
         <v>5</v>
@@ -8221,7 +8221,7 @@
         <v>46</v>
       </c>
       <c r="J104" s="0">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="K104" s="0">
         <v>21</v>
@@ -8233,16 +8233,16 @@
         <v>18</v>
       </c>
       <c r="N104" s="0">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="O104" s="0">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="P104" s="0">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="Q104" s="0">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="R104" s="0">
         <v>24</v>
@@ -8251,13 +8251,13 @@
         <v>25</v>
       </c>
       <c r="T104" s="0">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="U104" s="0">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="V104" s="0">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="W104" s="0">
         <v>16</v>

</xml_diff>